<commit_message>
equivalentes a dos pasadas de db:importar
</commit_message>
<xml_diff>
--- a/docs/formato-importacion-full.xlsx
+++ b/docs/formato-importacion-full.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\gestor-de-tareas\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF65F5A2-4612-4F07-85E2-4E5841E98BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="formato-importacion" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="44">
   <si>
     <t>kit</t>
   </si>
@@ -157,8 +156,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1014,23 +1013,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="51.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" customWidth="1"/>
-    <col min="9" max="9" width="17.7109375" customWidth="1"/>
-    <col min="10" max="10" width="30.5703125" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1062,7 +1061,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1090,8 +1089,11 @@
       <c r="I2">
         <v>1000</v>
       </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1119,8 +1121,11 @@
       <c r="I3">
         <v>1000</v>
       </c>
+      <c r="J3" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1148,8 +1153,11 @@
       <c r="I4">
         <v>1000</v>
       </c>
+      <c r="J4" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1177,8 +1185,11 @@
       <c r="I5">
         <v>1000</v>
       </c>
+      <c r="J5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1206,8 +1217,11 @@
       <c r="I6">
         <v>1000</v>
       </c>
+      <c r="J6" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1239,7 +1253,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1271,7 +1285,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -1303,7 +1317,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1332,7 +1346,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1364,7 +1378,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -1396,7 +1410,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
1.5.133: asignar en el kanban: corrigiendo la asignacion de tareas
</commit_message>
<xml_diff>
--- a/docs/formato-importacion-full.xlsx
+++ b/docs/formato-importacion-full.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\gestor-de-tareas\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98ACA347-D2EF-4975-84FE-FBDABA56F05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="formato-importacion" sheetId="1" r:id="rId1"/>
@@ -156,8 +157,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1013,23 +1014,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="51.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="24.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +1062,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1093,7 +1094,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1125,7 +1126,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1157,7 +1158,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1189,7 +1190,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1221,7 +1222,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1253,7 +1254,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1285,7 +1286,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -1317,7 +1318,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1346,7 +1347,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1378,7 +1379,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -1410,7 +1411,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>33</v>
       </c>

</xml_diff>